<commit_message>
feat(03-02): integrate assignment and status lifecycle into workbook
- Add Assignment Tracker sheet with tblAssignmentTracker to create_workbook.py
- Add frmAssignment UserForm creation (team/person cascade, incident list)
- Add frmStatusUpdate UserForm creation (status transitions, reason field)
- Extend inject_vba.py: 9 modules, 3 UserForms, 3 Dashboard buttons, 1 Refresh button
- Regenerate BRIMIS_IMS.xlsm with all Phase 3 components (114.8 KB, 13 VBA components)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BRIMIS_IMS.xlsx
+++ b/BRIMIS_IMS.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Tracker" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -274,6 +275,23 @@
     <tableColumn id="3" name="3-High"/>
     <tableColumn id="4" name="2-Medium"/>
     <tableColumn id="5" name="1-Low"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="tblAssignmentTracker" displayName="tblAssignmentTracker" ref="A2:H3" headerRowCount="1">
+  <autoFilter ref="A2:H3"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="AssignedTeam"/>
+    <tableColumn id="2" name="AssignedTo"/>
+    <tableColumn id="3" name="IncidentID"/>
+    <tableColumn id="4" name="Title"/>
+    <tableColumn id="5" name="Priority"/>
+    <tableColumn id="6" name="Status"/>
+    <tableColumn id="7" name="AssignedDate"/>
+    <tableColumn id="8" name="DaysOpen"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1467,4 +1485,92 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0032373C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>BRIMIS IMS - Assignment Tracker</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>AssignedTeam</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>AssignedTo</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>IncidentID</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>AssignedDate</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>DaysOpen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(06-02): regenerate workbook with search form and report template (191 KB)
- 13 VBA modules, 4 UserForms (frmSearch new), Dashboard sheet code
- 5 Dashboard buttons: Log, Assign, Update Status, Refresh, Search Incidents
- IncidentReport template sheet (VeryHidden) with BRIMIS-branded layout
- frmSearch: 30 controls (8 criteria, ListBox, 5 detail labels, 3 action buttons)
- File size grew from 160 KB to 191 KB with Phase 6 additions

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BRIMIS_IMS.xlsx
+++ b/BRIMIS_IMS.xlsx
@@ -12,8 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignment Tracker" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RCA Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IncidentReport" sheetId="6" state="veryHidden" r:id="rId6"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'IncidentReport'!$A$1:$H$35</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -100,6 +103,23 @@
       <color rgb="00808080"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00EE3124"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00EE3124"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0032373C"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -151,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -196,6 +216,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1969,4 +1999,267 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>BRIMIS</t>
+        </is>
+      </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>INCIDENT REPORT</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>Report Date:</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="D2" s="22" t="inlineStr">
+        <is>
+          <t>BRIMIS Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>INCIDENT OVERVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Incident ID:</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>Status:</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Title:</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Priority:</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>Category:</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Subcategory:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>DESCRIPTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="n"/>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>TIMELINE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Reported:</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>By:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Assigned:</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>To:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>Response:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Resolution:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>Closed:</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>ASSIGNMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Team:</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>Assigned To:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>Assigned Date:</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>Assigned By:</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>RESOLUTION &amp; ROOT CAUSE ANALYSIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>Root Cause:</t>
+        </is>
+      </c>
+      <c r="B28" s="25" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Corrective Action:</t>
+        </is>
+      </c>
+      <c r="B29" s="25" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>Preventive Action:</t>
+        </is>
+      </c>
+      <c r="B30" s="25" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
+          <t>Resolution Notes:</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>SLA PERFORMANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>Response SLA:</t>
+        </is>
+      </c>
+      <c r="D34" s="24" t="inlineStr">
+        <is>
+          <t>Resolution SLA:</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A11:H14"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="B28:H28"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>